<commit_message>
Add contribution tracker link to README
</commit_message>
<xml_diff>
--- a/docs/contribution_tracker.xlsx
+++ b/docs/contribution_tracker.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H3" s="16" t="n"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H9" s="16" t="n"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" s="16" t="n"/>
@@ -935,7 +935,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H12" s="16" t="n"/>
@@ -971,7 +971,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H13" s="16" t="n"/>

</xml_diff>